<commit_message>
Meal Plans Module Complete
</commit_message>
<xml_diff>
--- a/public/assets/excel/meal_plans.xlsx
+++ b/public/assets/excel/meal_plans.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo LOQ\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45B7E59-6446-4495-8F3D-B02921E5C4BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14614939-D16B-41C7-AA9B-CC9FB65F3701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -43,18 +43,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Breakfast</t>
-  </si>
-  <si>
-    <t>Lunch</t>
-  </si>
-  <si>
-    <t>Snacks</t>
-  </si>
-  <si>
-    <t>Dinner</t>
-  </si>
-  <si>
     <t>Paratha with egg</t>
   </si>
   <si>
@@ -91,9 +79,6 @@
     <t>7:45 PM</t>
   </si>
   <si>
-    <t>Active</t>
-  </si>
-  <si>
     <t>Sokal Nasta</t>
   </si>
   <si>
@@ -104,13 +89,28 @@
   </si>
   <si>
     <t>Raat er Kabar</t>
+  </si>
+  <si>
+    <t>breakfast</t>
+  </si>
+  <si>
+    <t>lunch</t>
+  </si>
+  <si>
+    <t>snacks</t>
+  </si>
+  <si>
+    <t>dinner</t>
+  </si>
+  <si>
+    <t>active</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,6 +122,21 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -162,11 +177,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -185,9 +202,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -225,9 +242,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -260,9 +277,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -295,9 +329,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -472,22 +523,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -502,103 +553,104 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>15</v>
-      </c>
-      <c r="E2" t="s">
-        <v>19</v>
       </c>
       <c r="F2">
         <v>25</v>
       </c>
-      <c r="G2" t="s">
-        <v>23</v>
+      <c r="G2" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>20</v>
       </c>
       <c r="F3">
         <v>80</v>
       </c>
-      <c r="G3" t="s">
-        <v>23</v>
+      <c r="G3" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>17</v>
-      </c>
-      <c r="E4" t="s">
-        <v>21</v>
       </c>
       <c r="F4">
         <v>25</v>
       </c>
-      <c r="G4" t="s">
-        <v>23</v>
+      <c r="G4" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>18</v>
-      </c>
-      <c r="E5" t="s">
-        <v>22</v>
       </c>
       <c r="F5">
         <v>70</v>
       </c>
-      <c r="G5" t="s">
-        <v>23</v>
+      <c r="G5" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>